<commit_message>
integracao da base de conhecimento
</commit_message>
<xml_diff>
--- a/relatorios/relatorio_faturamento_2024-01-01_a_2024-12-31.xlsx
+++ b/relatorios/relatorio_faturamento_2024-01-01_a_2024-12-31.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D175"/>
+  <dimension ref="A1:D199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1502,7 +1502,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1511,16 +1511,16 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1529,16 +1529,16 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1547,16 +1547,16 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1565,16 +1565,16 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1583,16 +1583,16 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1601,16 +1601,16 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1619,16 +1619,16 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1637,10 +1637,10 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="68">
@@ -2546,7 +2546,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -2555,16 +2555,16 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D118" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -2573,16 +2573,16 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D119" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -2591,16 +2591,16 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D120" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -2609,16 +2609,16 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D121" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -2627,16 +2627,16 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D122" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -2645,16 +2645,16 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D123" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -2663,16 +2663,16 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D124" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -2681,16 +2681,16 @@
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -2699,16 +2699,16 @@
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D126" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -2717,16 +2717,16 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D127" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -2735,16 +2735,16 @@
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D128" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -2753,16 +2753,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D129" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -2771,16 +2771,16 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D130" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -2789,16 +2789,16 @@
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D131" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -2807,16 +2807,16 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D132" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -2825,10 +2825,10 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D133" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="134">
@@ -3584,6 +3584,438 @@
         <v>2000</v>
       </c>
       <c r="D175" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D176" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D177" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D178" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D179" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D180" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D181" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D182" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D183" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D184" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C185" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D185" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D186" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D187" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D188" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D189" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D190" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D191" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D192" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C193" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D193" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D194" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D195" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D196" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D197" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D198" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D199" s="2" t="n">
         <v>45352</v>
       </c>
     </row>
@@ -3655,7 +4087,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C2" t="n">
         <v>1000</v>
@@ -3686,7 +4118,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C3" t="n">
         <v>1500</v>
@@ -3717,7 +4149,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C4" t="n">
         <v>2000</v>

</xml_diff>

<commit_message>
teste com nova funcionalidade
</commit_message>
<xml_diff>
--- a/relatorios/relatorio_faturamento_2024-01-01_a_2024-12-31.xlsx
+++ b/relatorios/relatorio_faturamento_2024-01-01_a_2024-12-31.xlsx
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D199"/>
+  <dimension ref="A1:D211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1646,7 +1646,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1655,16 +1655,16 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1673,16 +1673,16 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1691,16 +1691,16 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Unidade B</t>
+          <t>Unidade A</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1709,10 +1709,10 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1500</v>
+        <v>1000</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>45323</v>
+        <v>45292</v>
       </c>
     </row>
     <row r="72">
@@ -2834,7 +2834,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -2843,16 +2843,16 @@
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D134" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -2861,16 +2861,16 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D135" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -2879,16 +2879,16 @@
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D136" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -2897,16 +2897,16 @@
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D137" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -2915,16 +2915,16 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D138" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -2933,16 +2933,16 @@
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D139" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -2951,16 +2951,16 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D140" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Unidade C</t>
+          <t>Unidade B</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -2969,10 +2969,10 @@
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="D141" s="2" t="n">
-        <v>45352</v>
+        <v>45323</v>
       </c>
     </row>
     <row r="142">
@@ -4016,6 +4016,222 @@
         <v>2000</v>
       </c>
       <c r="D199" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D200" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D201" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C202" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D202" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D203" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D204" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D205" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D206" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D207" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D208" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D209" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D210" s="2" t="n">
+        <v>45352</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Unidade C</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Faturamento</t>
+        </is>
+      </c>
+      <c r="C211" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D211" s="2" t="n">
         <v>45352</v>
       </c>
     </row>
@@ -4087,7 +4303,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C2" t="n">
         <v>1000</v>
@@ -4118,7 +4334,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C3" t="n">
         <v>1500</v>
@@ -4149,7 +4365,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C4" t="n">
         <v>2000</v>

</xml_diff>